<commit_message>
feat: add beta notice modal, update Excel export template, fix role management, and optimize page performance
</commit_message>
<xml_diff>
--- a/public/gradebook-templates/both-terms.xlsx
+++ b/public/gradebook-templates/both-terms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jks20\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D650578F-441D-47F8-B877-8C5582558E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F087A9-4B5F-425A-AA1C-47EFD0451271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -515,7 +515,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -540,10 +540,88 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -552,89 +630,14 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1037,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr defaultRowHeight="19.95" customHeight="1" x14ac:dyDescent="0.65"/>
   <cols>
     <col min="1" max="1" width="7.796875" style="2" customWidth="1"/>
@@ -1050,185 +1053,185 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="H1" s="33"/>
-      <c r="J1" s="33"/>
+      <c r="H1" s="10"/>
+      <c r="J1" s="10"/>
     </row>
     <row r="2" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="H2" s="33"/>
-      <c r="J2" s="33"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="H2" s="10"/>
+      <c r="J2" s="10"/>
     </row>
     <row r="3" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="38" t="s">
+      <c r="C3" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="H3" s="33"/>
-      <c r="J3" s="33"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="H3" s="10"/>
+      <c r="J3" s="10"/>
     </row>
     <row r="4" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="H4" s="33"/>
-      <c r="J4" s="33"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="H4" s="10"/>
+      <c r="J4" s="10"/>
     </row>
     <row r="5" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="10" t="s">
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="32" t="s">
+      <c r="K6" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="10" t="s">
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="32" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="35"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="41" t="s">
+      <c r="A7" s="12"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15" t="s">
+      <c r="G7" s="31"/>
+      <c r="H7" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="16"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="13" t="s">
+      <c r="I7" s="29"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="14"/>
-      <c r="M7" s="15" t="s">
+      <c r="L7" s="31"/>
+      <c r="M7" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="N7" s="16"/>
-      <c r="O7" s="11"/>
+      <c r="N7" s="29"/>
+      <c r="O7" s="33"/>
     </row>
     <row r="8" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A8" s="35"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="39">
+      <c r="A8" s="12"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="26">
         <v>40</v>
       </c>
-      <c r="G8" s="40"/>
-      <c r="H8" s="19">
+      <c r="G8" s="27"/>
+      <c r="H8" s="24">
         <v>20</v>
       </c>
-      <c r="I8" s="20"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="17">
+      <c r="I8" s="25"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="40">
         <v>40</v>
       </c>
-      <c r="L8" s="18"/>
-      <c r="M8" s="19">
+      <c r="L8" s="41"/>
+      <c r="M8" s="24">
         <v>20</v>
       </c>
-      <c r="N8" s="20"/>
-      <c r="O8" s="11"/>
+      <c r="N8" s="25"/>
+      <c r="O8" s="33"/>
     </row>
     <row r="9" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="35"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="21" t="s">
+      <c r="A9" s="12"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="25" t="s">
+      <c r="H9" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="27" t="s">
+      <c r="I9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="11"/>
-      <c r="K9" s="21" t="s">
+      <c r="J9" s="33"/>
+      <c r="K9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="M9" s="25" t="s">
+      <c r="M9" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="N9" s="27" t="s">
+      <c r="N9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="11"/>
+      <c r="O9" s="33"/>
     </row>
     <row r="10" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="36"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="29"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="26"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="12"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="38"/>
     </row>
     <row r="11" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A11" s="6">
@@ -1405,7 +1408,7 @@
       <c r="O20" s="4"/>
     </row>
     <row r="21" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A21" s="8">
+      <c r="A21" s="6">
         <v>11</v>
       </c>
       <c r="B21" s="3"/>
@@ -1477,7 +1480,7 @@
       <c r="O24" s="4"/>
     </row>
     <row r="25" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A25" s="6">
+      <c r="A25" s="8">
         <v>15</v>
       </c>
       <c r="B25" s="3"/>
@@ -1513,7 +1516,7 @@
       <c r="O26" s="4"/>
     </row>
     <row r="27" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A27" s="8">
+      <c r="A27" s="6">
         <v>17</v>
       </c>
       <c r="B27" s="3"/>
@@ -1621,7 +1624,7 @@
       <c r="O32" s="4"/>
     </row>
     <row r="33" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A33" s="8">
+      <c r="A33" s="6">
         <v>23</v>
       </c>
       <c r="B33" s="3"/>
@@ -1657,7 +1660,7 @@
       <c r="O34" s="4"/>
     </row>
     <row r="35" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A35" s="6">
+      <c r="A35" s="8">
         <v>25</v>
       </c>
       <c r="B35" s="3"/>
@@ -1692,8 +1695,204 @@
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
     </row>
+    <row r="37" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A37" s="6">
+        <v>27</v>
+      </c>
+      <c r="J37" s="4"/>
+      <c r="O37" s="4"/>
+    </row>
+    <row r="38" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="7">
+        <v>28</v>
+      </c>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="4"/>
+      <c r="O38" s="4"/>
+    </row>
+    <row r="39" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A39" s="6">
+        <v>29</v>
+      </c>
+      <c r="J39" s="4"/>
+      <c r="O39" s="4"/>
+    </row>
+    <row r="40" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7">
+        <v>30</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+    </row>
+    <row r="41" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A41" s="6">
+        <v>31</v>
+      </c>
+      <c r="J41" s="4"/>
+      <c r="O41" s="4"/>
+    </row>
+    <row r="42" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7">
+        <v>32</v>
+      </c>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+    </row>
+    <row r="43" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A43" s="6">
+        <v>33</v>
+      </c>
+      <c r="J43" s="4"/>
+      <c r="O43" s="4"/>
+    </row>
+    <row r="44" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7">
+        <v>34</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+    </row>
+    <row r="45" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A45" s="8">
+        <v>35</v>
+      </c>
+      <c r="J45" s="4"/>
+      <c r="O45" s="4"/>
+    </row>
+    <row r="46" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="7">
+        <v>36</v>
+      </c>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+    </row>
+    <row r="47" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A47" s="6">
+        <v>37</v>
+      </c>
+      <c r="J47" s="4"/>
+      <c r="O47" s="4"/>
+    </row>
+    <row r="48" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7">
+        <v>38</v>
+      </c>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+    </row>
+    <row r="49" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="A49" s="42">
+        <v>39</v>
+      </c>
+      <c r="J49" s="4"/>
+      <c r="O49" s="4"/>
+    </row>
+    <row r="50" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="6">
+        <v>40</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="O6:O10"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="C6:C10"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="J6:J10"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="K6:N6"/>
     <mergeCell ref="J1:J4"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="C2:F2"/>
@@ -1710,20 +1909,6 @@
     <mergeCell ref="H1:H4"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="D6:D10"/>
-    <mergeCell ref="C6:C10"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="J6:J10"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="O6:O10"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="N9:N10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>